<commit_message>
temp: Splitter-Fix (locale-feste Kriterien)
</commit_message>
<xml_diff>
--- a/x/u29xk/expense-splitter/Shared-Expense-Splitter.xlsx
+++ b/x/u29xk/expense-splitter/Shared-Expense-Splitter.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fabianhones/Desktop/Geld_verdienen/experiment/products/expense-splitter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1AEC116-08C5-C648-8618-246C7EAF8F3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90DA64B1-8079-A54C-BBB4-2E1C45D08B0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28352,12 +28352,12 @@
         <v>1000.37</v>
       </c>
       <c r="E5" s="36">
-        <f>IF($J$1=0,"—",IFERROR(ROUND(SUMIF($F$10:$F$19,"&gt;0.009"),2),0))</f>
-        <v>0</v>
+        <f>IF($J$1=0,"—",IFERROR(ROUND(SUMIF($F$10:$F$19,"&gt;"&amp;0.009),2),0))</f>
+        <v>1659.04</v>
       </c>
       <c r="F5" s="37">
-        <f>IF($J$1=0,"—",IFERROR(COUNTIF('Settle Up'!$V$10:$V$18,"&gt;=0.01"),0))</f>
-        <v>0</v>
+        <f>IF($J$1=0,"—",IFERROR(COUNTIF('Settle Up'!$V$10:$V$18,"&gt;="&amp;0.01),0))</f>
+        <v>4</v>
       </c>
       <c r="G5" s="37" t="str">
         <f>IF($J$1=0,"—",IF(SUMPRODUCT((Setup!$G$21:$G$30&lt;&gt;"")*1)&gt;0,"Duplicate member name on Setup — give every member a unique name",IF(COUNTIF(Expenses!$R$8:$R$307,"OK")=$J$1,"All good","Fix "&amp;($J$1-COUNTIF(Expenses!$R$8:$R$307,"OK"))&amp;" row(s) — see Check column")))</f>
@@ -28914,8 +28914,8 @@
     </row>
     <row r="4" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="59" t="str">
-        <f>IF('Who Owes What'!$J$1=0,"Nothing logged yet — start on the Expenses sheet.",IF(AND(ISNUMBER('Who Owes What'!$F$20),ABS('Who Owes What'!$F$20)&gt;0.01),"⚠ Fix the flagged rows on the Expenses sheet first — the balances do not add up to 0.",IF(COUNTIF($V$10:$V$18,"&gt;=0.01")=0,"Nothing to settle — everyone is square.",COUNTIF($V$10:$V$18,"&gt;=0.01")&amp;" transfer(s) clear all balances. Tick them off in 'Done?'.")))</f>
-        <v>Nothing to settle — everyone is square.</v>
+        <f>IF('Who Owes What'!$J$1=0,"Nothing logged yet — start on the Expenses sheet.",IF(AND(ISNUMBER('Who Owes What'!$F$20),ABS('Who Owes What'!$F$20)&gt;0.01),"⚠ Fix the flagged rows on the Expenses sheet first — the balances do not add up to 0.",IF(COUNTIF($V$10:$V$18,"&gt;="&amp;0.01)=0,"Nothing to settle — everyone is square.",COUNTIF($V$10:$V$18,"&gt;="&amp;0.01)&amp;" transfer(s) clear all balances. Tick them off in 'Done?'.")))</f>
+        <v>4 transfer(s) clear all balances. Tick them off in 'Done?'.</v>
       </c>
       <c r="C4" s="52"/>
       <c r="D4" s="52"/>
@@ -29781,7 +29781,7 @@
         <v>143</v>
       </c>
       <c r="E20" s="49">
-        <f>IF('Who Owes What'!$J$1=0,"—",IFERROR(ROUND(MAX(SUMIF($J$19:$S$19,"&gt;0.009"),-SUMIF($J$19:$S$19,"&lt;-0.009")),2),0))</f>
+        <f>IF('Who Owes What'!$J$1=0,"—",IFERROR(ROUND(MAX(SUMIF($J$19:$S$19,"&gt;"&amp;0.009),-SUMIF($J$19:$S$19,"&lt;-0.009")),2),0))</f>
         <v>0</v>
       </c>
     </row>
@@ -29790,8 +29790,8 @@
         <v>144</v>
       </c>
       <c r="E21" s="49">
-        <f>IF('Who Owes What'!$J$1=0,"—",IFERROR(SUMIF($V$10:$V$18,"&gt;=0.01"),0))</f>
-        <v>0</v>
+        <f>IF('Who Owes What'!$J$1=0,"—",IFERROR(SUMIF($V$10:$V$18,"&gt;="&amp;0.01),0))</f>
+        <v>1659.04</v>
       </c>
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.2">
@@ -29799,8 +29799,8 @@
         <v>145</v>
       </c>
       <c r="E22" s="50" t="str">
-        <f>IF(COUNTIF($V$10:$V$18,"&gt;=0.01")=0,"—",COUNTIF($F$10:$F$18,"Yes")&amp;" of "&amp;COUNTIF($V$10:$V$18,"&gt;=0.01")&amp;" done")</f>
-        <v>—</v>
+        <f>IF(COUNTIF($V$10:$V$18,"&gt;="&amp;0.01)=0,"—",COUNTIF($F$10:$F$18,"Yes")&amp;" of "&amp;COUNTIF($V$10:$V$18,"&gt;="&amp;0.01)&amp;" done")</f>
+        <v>0 of 4 done</v>
       </c>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.2">

</xml_diff>